<commit_message>
Agrega hojas de respuestas con gráficos al Excel de práctica
Mantiene las 4 hojas de ejercicios en blanco y suma 4 hojas de respuestas
(estilo plano) con todo resuelto, los gráficos y la interpretación:
- Ingreso: curva de ingreso (loma) y de demanda; óptimo en P=5.
- Producción: PT y PM/Pme; óptimo técnico en L=5.
- Costos económicos: contable/oportunidad/económico.
- Costos: CM y CTMe; escala eficiente (mínimo CTMe) en q=7.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JHgctdgkpncN2RzQexXhAR
</commit_message>
<xml_diff>
--- a/economia-practica.xlsx
+++ b/economia-practica.xlsx
@@ -11,6 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Producción CP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Costos económicos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Costos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Ingreso (resp)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Producción (resp)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Costos econ (resp)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Costos (resp)" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0#"/>
+    <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +50,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +70,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -106,17 +125,52 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -191,6 +245,793 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Curva de ingreso total (loma)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>IT</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'1. Ingreso (resp)'!$B$6:$B$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'1. Ingreso (resp)'!$C$6:$C$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cantidad</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>IT ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Curva de demanda</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Precio</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'1. Ingreso (resp)'!$B$6:$B$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'1. Ingreso (resp)'!$A$6:$A$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cantidad</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Precio</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Producto total (PT)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>PT</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'2. Producción (resp)'!$A$5:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2. Producción (resp)'!$B$5:$B$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>L</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Producto</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>PM y Pme</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>PM</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'2. Producción (resp)'!$A$6:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2. Producción (resp)'!$C$6:$C$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Pme</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'2. Producción (resp)'!$A$6:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2. Producción (resp)'!$D$6:$D$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>L</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Producto</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Costo marginal (CM) y total medio (CTMe)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>CM</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'4. Costos (resp)'!$A$6:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'4. Costos (resp)'!$E$6:$E$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>CTMe</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'4. Costos (resp)'!$A$6:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'4. Costos (resp)'!$F$6:$F$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>q</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>$</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -482,11 +1323,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -547,141 +1388,133 @@
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Ejercicio 2: Dados los siguientes datos:</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>a) Calcular el ingreso total.   b) Observar la tabla e interpretar, relacionando el precio con el ingreso.   c) Graficar la curva de demanda y la curva de ingreso.   d) Interpretar los gráficos y marcar el óptimo.</t>
+          <t>Ejercicio 2: a) Calcular el ingreso total.  b) Interpretar relacionando el precio con el ingreso.  c) Graficar la curva de demanda y la de ingreso.  d) Interpretar y marcar el óptimo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>IT = P·Q</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>IT = P·Q</t>
-        </is>
-      </c>
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B15" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B16" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B17" s="4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="C17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B18" s="4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" s="4" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" s="4" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="4" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="C21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" s="4" t="n">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="C22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" s="4" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C23" s="5" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="C24" s="5" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A10:H10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -694,13 +1527,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -720,7 +1553,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>b) Graficar la curva de producto total, marginal y medio. Marcar el óptimo técnico. Describir el comportamiento de las curvas.</t>
+          <t>b) Graficar la curva de producto total, marginal y medio. Marcar el óptimo técnico y describir el comportamiento de las curvas.</t>
         </is>
       </c>
     </row>
@@ -858,8 +1691,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -871,7 +1704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -885,10 +1718,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="55" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Un pequeño fabricante de helado desembolsa $70.000 por mes para pagar las materias primas y $50.000 para el sueldo de un empleado. Como usa un local de su propiedad no paga alquiler, pero otras empresas pagan $30.000 por locales similares. Además, si se emplease como electricista (su profesión) ganaría $200.000 al mes.</t>
+          <t>Un fabricante de helado paga $70.000 de materias primas y $50.000 de sueldo. Usa un local propio (no paga alquiler, pero otros pagan $30.000 por locales similares). Si trabajara de electricista (su profesión) ganaría $200.000 al mes.</t>
         </is>
       </c>
     </row>
@@ -965,8 +1798,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -982,13 +1815,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1001,14 +1834,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>a) Calcular el costo total, costo marginal, costo total medio, costo fijo medio y costo variable medio.</t>
+          <t>a) Calcular el costo total (CT), costo marginal (CM), costo total medio (CTMe), costo fijo medio (CFMe) y costo variable medio (CVMe).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>b) Graficar la curva de costo marginal (CM) y costo total medio (CTMe) e identificar el nivel de producción que minimiza los costos.</t>
+          <t>b) Graficar la curva de CM y CTMe e identificar el nivel de producción que minimiza los costos.</t>
         </is>
       </c>
     </row>
@@ -1237,4 +2070,904 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RESPUESTA — Ingreso total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Ej.1: a P=10 → Q=500, IT=5000 (elasticidad unitaria).  A P=12 → Q=400, IT=4800 (elástica).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>IT = P·Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>INTERPRETACIÓN: cuando el precio baja, el IT sube hasta su máximo en P=$5 (Q=100, IT=$500); por debajo de $5 el IT baja. En P=$5 la elasticidad es unitaria y ahí se maximiza el ingreso. La curva de IT sube, llega al óptimo y desciende.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A18:H20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RESPUESTA — Producción en el corto plazo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Pme</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>136</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>83.33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>381</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>131</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>95.25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>580</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>96.67</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>653</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>73</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>93.29000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>695</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>86.88</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>720</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>720</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>INTERPRETACIÓN: el PT crece, tiene un punto de inflexión en el 4º trabajador. El PM crece hasta el 4º trabajador y luego decrece hasta hacerse nulo (L=10). El Pme aumenta y desde el 5º trabajador decrece: ahí está el ÓPTIMO TÉCNICO (PM corta al Pme en su máximo). Cuando PM&gt;Pme el Pme sube; cuando PM&lt;Pme el Pme baja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A17:H19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RESPUESTA — Costo contable, de oportunidad y económico</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Materias primas (paga)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Sueldo del empleado (paga)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Alquiler que no cobra</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Sueldo de electricista que resigna</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Costo CONTABLE (70.000+50.000)</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Costo de OPORTUNIDAD (30.000+200.000)</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Costo ECONÓMICO (120.000+230.000)</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>INTERPRETACIÓN: el contador solo cuenta los $120.000 que se pagan (explícitos). El economista suma lo que se resigna (alquiler no cobrado + sueldo de electricista = $230.000), por eso el costo económico es $350.000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:H15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RESPUESTA — Familia de costos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PT (Q)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>CTMe</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>CFMe</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>CVMe</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>24.38</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>13.12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>20.42</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>12.92</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>93.7</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <v>138.7</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>13.39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>160</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>14.38</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>143.7</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>188.7</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>15.97</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>177.5</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>222.5</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>q que minimiza el CTMe = 7  (CTMe ≈ 19.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>INTERPRETACIÓN: el CTMe se minimiza en q=7 (≈19,8): ese punto, donde el CM corta al CTMe, se llama ESCALA EFICIENTE (la cantidad que minimiza el costo total medio). Antes el CTMe baja, después sube; el CFMe siempre baja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A19:H21"/>
+    <mergeCell ref="A17:E17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Completa la respuesta del Ejercicio 1 de Ingreso total (IT y elasticidad)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JHgctdgkpncN2RzQexXhAR
</commit_message>
<xml_diff>
--- a/economia-practica.xlsx
+++ b/economia-practica.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="0.0#"/>
     <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,13 @@
     <font/>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
     <font>
       <i val="1"/>
@@ -109,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,18 +143,20 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -291,12 +300,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'1. Ingreso (resp)'!$B$6:$B$16</f>
+              <f>'1. Ingreso (resp)'!$B$17:$B$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'1. Ingreso (resp)'!$C$6:$C$16</f>
+              <f>'1. Ingreso (resp)'!$C$17:$C$27</f>
             </numRef>
           </val>
         </ser>
@@ -411,12 +420,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'1. Ingreso (resp)'!$B$6:$B$16</f>
+              <f>'1. Ingreso (resp)'!$B$17:$B$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'1. Ingreso (resp)'!$A$6:$A$16</f>
+              <f>'1. Ingreso (resp)'!$A$17:$A$27</f>
             </numRef>
           </val>
         </ser>
@@ -915,7 +924,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="3060000"/>
@@ -937,7 +946,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="3060000"/>
@@ -2078,12 +2087,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2096,161 +2106,242 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Ej.1: a P=10 → Q=500, IT=5000 (elasticidad unitaria).  A P=12 → Q=400, IT=4800 (elástica).</t>
+          <t>Ejercicio 1:  Q = 1000 − 50·P</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Q = 1000−50P</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>IT = P·Q</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>IT = P·Q</t>
-        </is>
+      <c r="A5" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Elasticidad-precio (variación % desde el punto de partida):</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>•  En P=$10:   Ep = |(−100/500) / (2/10)| = 1   →   UNITARIA  (ahí el IT es máximo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>•  En P=$12:   Ep = |(100/400) / (−2/12)| = 1,5   →   ELÁSTICA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>INTERPRETACIÓN: en P=$10 la elasticidad es unitaria y se obtiene el mayor ingreso total. Partiendo de P=$12 la demanda es elástica, por lo cual al BAJAR el precio (de $12 a $10) el ingreso total SUBE (de $4.800 a $5.000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Ejercicio 2:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>IT = P·Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C17" s="11" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+    <row r="18">
+      <c r="A18" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B18" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C18" s="11" t="n">
         <v>180</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="19">
+      <c r="A19" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B19" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C19" s="11" t="n">
         <v>320</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+    <row r="20">
+      <c r="A20" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B20" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C20" s="11" t="n">
         <v>420</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+    <row r="21">
+      <c r="A21" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B21" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C21" s="11" t="n">
         <v>480</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="n">
+    <row r="22">
+      <c r="A22" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B22" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C22" s="16" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+    <row r="23">
+      <c r="A23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B23" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C23" s="11" t="n">
         <v>480</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
+    <row r="24">
+      <c r="A24" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B24" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C24" s="11" t="n">
         <v>420</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+    <row r="25">
+      <c r="A25" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B25" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C25" s="11" t="n">
         <v>320</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
+    <row r="26">
+      <c r="A26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B26" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C26" s="11" t="n">
         <v>180</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+    <row r="27">
+      <c r="A27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B27" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C27" s="11" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>INTERPRETACIÓN: cuando el precio baja, el IT sube hasta su máximo en P=$5 (Q=100, IT=$500); por debajo de $5 el IT baja. En P=$5 la elasticidad es unitaria y ahí se maximiza el ingreso. La curva de IT sube, llega al óptimo y desciende.</t>
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
+    <row r="30"/>
+    <row r="31"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A18:H20"/>
+  <mergeCells count="7">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A11:H13"/>
+    <mergeCell ref="A29:H31"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A8:H8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2326,10 +2417,10 @@
       <c r="B6" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="17" t="n">
         <v>55</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="17" t="n">
         <v>55</v>
       </c>
     </row>
@@ -2340,10 +2431,10 @@
       <c r="B7" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="17" t="n">
         <v>59</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="17" t="n">
         <v>57</v>
       </c>
     </row>
@@ -2354,10 +2445,10 @@
       <c r="B8" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="17" t="n">
         <v>136</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="17" t="n">
         <v>83.33</v>
       </c>
     </row>
@@ -2368,24 +2459,24 @@
       <c r="B9" s="4" t="n">
         <v>381</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="17" t="n">
         <v>131</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="17" t="n">
         <v>95.25</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="15" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>500</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="18" t="n">
         <v>119</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="19" t="n">
         <v>100</v>
       </c>
     </row>
@@ -2396,10 +2487,10 @@
       <c r="B11" s="4" t="n">
         <v>580</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="17" t="n">
         <v>80</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="17" t="n">
         <v>96.67</v>
       </c>
     </row>
@@ -2410,10 +2501,10 @@
       <c r="B12" s="4" t="n">
         <v>653</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="17" t="n">
         <v>73</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="17" t="n">
         <v>93.29000000000001</v>
       </c>
     </row>
@@ -2424,10 +2515,10 @@
       <c r="B13" s="4" t="n">
         <v>695</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="17" t="n">
         <v>42</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="17" t="n">
         <v>86.88</v>
       </c>
     </row>
@@ -2438,10 +2529,10 @@
       <c r="B14" s="4" t="n">
         <v>720</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="17" t="n">
         <v>80</v>
       </c>
     </row>
@@ -2452,10 +2543,10 @@
       <c r="B15" s="4" t="n">
         <v>720</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="17" t="n">
         <v>72</v>
       </c>
     </row>
@@ -2543,7 +2634,7 @@
           <t>Costo CONTABLE (70.000+50.000)</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="20" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -2553,7 +2644,7 @@
           <t>Costo de OPORTUNIDAD (30.000+200.000)</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="20" t="n">
         <v>230000</v>
       </c>
     </row>
@@ -2563,7 +2654,7 @@
           <t>Costo ECONÓMICO (120.000+230.000)</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="20" t="n">
         <v>350000</v>
       </c>
     </row>
@@ -2662,7 +2753,7 @@
       <c r="C5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="21" t="n">
         <v>45</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2696,19 +2787,19 @@
       <c r="C6" s="9" t="n">
         <v>22.5</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="21" t="n">
         <v>67.5</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="21" t="n">
         <v>22.5</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="21" t="n">
         <v>67.5</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="21" t="n">
         <v>22.5</v>
       </c>
     </row>
@@ -2722,19 +2813,19 @@
       <c r="C7" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="21" t="n">
         <v>12.5</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="21" t="n">
         <v>22.5</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="21" t="n">
         <v>17.5</v>
       </c>
     </row>
@@ -2748,19 +2839,19 @@
       <c r="C8" s="9" t="n">
         <v>45</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="21" t="n">
         <v>90</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="21" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2774,19 +2865,19 @@
       <c r="C9" s="9" t="n">
         <v>52.5</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="21" t="n">
         <v>97.5</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="21" t="n">
         <v>7.5</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="21" t="n">
         <v>24.38</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="21" t="n">
         <v>11.25</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="21" t="n">
         <v>13.12</v>
       </c>
     </row>
@@ -2800,19 +2891,19 @@
       <c r="C10" s="9" t="n">
         <v>62.5</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="21" t="n">
         <v>107.5</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="21" t="n">
         <v>21.5</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="21" t="n">
         <v>12.5</v>
       </c>
     </row>
@@ -2826,24 +2917,24 @@
       <c r="C11" s="9" t="n">
         <v>77.5</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="21" t="n">
         <v>122.5</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="21" t="n">
         <v>20.42</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="21" t="n">
         <v>7.5</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="H11" s="21" t="n">
         <v>12.92</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="15" t="n">
         <v>7</v>
       </c>
       <c r="B12" s="4" t="n">
@@ -2852,19 +2943,19 @@
       <c r="C12" s="9" t="n">
         <v>93.7</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="22" t="n">
         <v>138.7</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="22" t="n">
         <v>16.2</v>
       </c>
-      <c r="F12" s="21" t="n">
+      <c r="F12" s="23" t="n">
         <v>19.81</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="22" t="n">
         <v>6.43</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="H12" s="22" t="n">
         <v>13.39</v>
       </c>
     </row>
@@ -2878,19 +2969,19 @@
       <c r="C13" s="9" t="n">
         <v>115</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="21" t="n">
         <v>160</v>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="21" t="n">
         <v>21.3</v>
       </c>
-      <c r="F13" s="19" t="n">
+      <c r="F13" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="G13" s="19" t="n">
+      <c r="G13" s="21" t="n">
         <v>5.62</v>
       </c>
-      <c r="H13" s="19" t="n">
+      <c r="H13" s="21" t="n">
         <v>14.38</v>
       </c>
     </row>
@@ -2904,19 +2995,19 @@
       <c r="C14" s="9" t="n">
         <v>143.7</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="21" t="n">
         <v>188.7</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="21" t="n">
         <v>28.7</v>
       </c>
-      <c r="F14" s="19" t="n">
+      <c r="F14" s="21" t="n">
         <v>20.97</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="21" t="n">
         <v>15.97</v>
       </c>
     </row>
@@ -2930,24 +3021,24 @@
       <c r="C15" s="9" t="n">
         <v>177.5</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="21" t="n">
         <v>222.5</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="21" t="n">
         <v>33.8</v>
       </c>
-      <c r="F15" s="19" t="n">
+      <c r="F15" s="21" t="n">
         <v>22.25</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="G15" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H15" s="21" t="n">
         <v>17.75</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>q que minimiza el CTMe = 7  (CTMe ≈ 19.81)</t>
         </is>

</xml_diff>

<commit_message>
Usa la fórmula de elasticidad de la cátedra en el Ej1 de ingreso
Ep = (%ΔQ)/(%ΔP), con %ΔQ=(Q1-Q0)/Q0 y %ΔP=(P1-P0)/P0, con el paso a paso.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JHgctdgkpncN2RzQexXhAR
</commit_message>
<xml_diff>
--- a/economia-practica.xlsx
+++ b/economia-practica.xlsx
@@ -1554,7 +1554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1626,40 +1626,42 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Elasticidad (variación % desde el punto de partida):</t>
+          <t>Fórmula (cátedra):   Ep = (%ΔQ) / (%ΔP) ,   con   %ΔQ = (Q1 − Q0)/Q0   y   %ΔP = (P1 − P0)/P0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>•  P=$10:  Ep = |(−100/500)/(2/10)| = 1  →  UNITARIA  (ahí el IT es máximo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>•  P=$12:  Ep = |(100/400)/(−2/12)| = 1,5  →  ELÁSTICA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+          <t>En P=$10  (P0=10 → P1=12):   %ΔQ = (400 − 500)/500 = -0,20 ;   %ΔP = (12 − 10)/10 = 0,20 ;   Ep = -0,20 / 0,20 = -1   →   |Ep| = 1   →   UNITARIA  (ahí el IT es máximo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>En P=$12  (P0=12 → P1=10):   %ΔQ = (500 − 400)/400 = 0,25 ;   %ΔP = (10 − 12)/12 = -0,167 ;   Ep = 0,25 / -0,167 = -1,5   →   |Ep| = 1,5   →   ELÁSTICA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>INTERPRETACIÓN: en P=$10 la elasticidad es unitaria y se obtiene el mayor ingreso total. Partiendo de P=$12 (zona elástica), al BAJAR el precio a $10 el ingreso total SUBE (de $4.800 a $5.000).</t>
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A11:J12"/>
+    <mergeCell ref="A16:J18"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A13:J14"/>
     <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A14:J16"/>
-    <mergeCell ref="A11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>